<commit_message>
Add author data to the OpenAlex pipeline
Extends fetch_openalex_works.py to pull authorships per work, storing both
the full author list and a display-truncated string (first + up to 4
middle + last) per the papers-table spec. Re-ran fetch + filter; same
27-work clean dataset, now with authors.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/openalex_works.xlsx
+++ b/data/openalex_works.xlsx
@@ -413,17 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,35 +435,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Authors</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Total citations</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Citations by year</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Not mine? (mark X)</t>
         </is>
@@ -474,33 +480,38 @@
           <t>The ProteomeXchange consortium in 2026: making proteomics data FAIR</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Eric W. Deutsch, Nuno Bandeira, Yasset Pérez‐Riverol, Vagisha Sharma, Jeremy Carver, ..., Juan Antonio Vizcaíno</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>2025</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Nucleic Acids Research</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/nar/gkaf1146</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>33</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2025: 2; 2026: 31</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -508,33 +519,38 @@
           <t>Comet Fragment-Ion Indexing for Enhanced Peptide Sequencing</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Christopher D. McGann, Erik J. Bergstrom, Vagisha Sharma, Lilian R. Heil, Qing Yu, ..., Devin K. Schweppe</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>2025</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.jproteome.4c01094</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026: 4</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -542,33 +558,38 @@
           <t>Comprehensive Proteomics Metadata and Integrative Web Portals Facilitate Sharing and Integration of LINCS Multiomics Data</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>D. Vidović, Behrouz Shamsaei, Stephan C. Schürer, Phillip Kogan, Szymon Chojnacki, ..., Michael J. MacCoss</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>2025</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Molecular &amp; Cellular Proteomics</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.mcpro.2025.100947</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026: 1</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -576,29 +597,34 @@
           <t>Corrigendum to “Comprehensive Proteomics Metadata and Integrative Web Portals Facilitate Sharing and Integration of LINCS Multiomics Data”</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D. Vidović, Behrouz Shamsaei, Stephan C. Schürer, Phillip Kogan, Szymon Chojnacki, ..., Michael J. MacCoss</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>2025</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>erratum</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Molecular &amp; Cellular Proteomics</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.mcpro.2025.100995</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -606,33 +632,38 @@
           <t>A Framework for Quality Control in Quantitative Proteomics</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kristine A. Tsantilas, Gennifer E. Merrihew, Julia Robbins, Richard S. Johnson, Jea Park, ..., Michael J. MacCoss</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>2024</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.jproteome.4c00363</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>28</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>2024: 3; 2025: 15; 2026: 10</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -640,33 +671,38 @@
           <t>A framework for quality control in quantitative proteomics</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kristine A. Tsantilas, Gennifer E. Merrihew, Julia Robbins, Richard S. Johnson, Jea Park, ..., Michael J. MacCoss</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>2024</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>bioRxiv (Cold Spring Harbor Laboratory)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://doi.org/10.1101/2024.04.12.589318</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>6</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>2024: 5; 2025: 1</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -674,33 +710,38 @@
           <t>Comet fragment-ion indexing for enhanced peptide sequencing</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Christopher D. McGann, Erik J. Bergstrom, Vagisha Sharma, Lilian R. Heil, Qing Yu, ..., Devin K. Schweppe</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>2024</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>bioRxiv (Cold Spring Harbor Laboratory)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1101/2024.10.11.617953</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>2</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>2025: 2</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -708,33 +749,38 @@
           <t>The ProteomeXchange consortium at 10 years: 2023 update</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Eric W. Deutsch, Nuno Bandeira, Yasset Pérez‐Riverol, Vagisha Sharma, Jeremy Carver, ..., Juan Antonio Vizcaíno</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>2022</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Nucleic Acids Research</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/nar/gkac1040</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>876</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>2022: 1; 2023: 142; 2024: 301; 2025: 296; 2026: 136</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -742,33 +788,38 @@
           <t>A Modified Feature Optimization Approach with Convolutional Neural Network for Apple Leaf Disease Detection</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Vagisha Sharma, Amandeep Verma, Neelam Goel</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>2022</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>conference-paper</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Lecture notes in networks and systems</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/978-3-030-96299-9_54</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>2</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>2022: 1; 2024: 1</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -776,33 +827,38 @@
           <t>Skyline Batch: An Intuitive User Interface for Batch Processing with Skyline</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Alexandra N. Marsh, Vagisha Sharma, Surya K. Mani, Olga Vitek, Michael J. MacCoss, Brendan MacLean</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>2021</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.jproteome.1c00749</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>9</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>2022: 1; 2023: 2; 2024: 4; 2025: 1; 2026: 1</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -810,33 +866,38 @@
           <t>Proteomic profiling dataset of chemical perturbations in multiple biological backgrounds</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Deborah Dele‐Oni, Karen E. Christianson, Shawn B. Egri, Alvaro Sebastian Vaca Jácome, Katherine C. DeRuff, ..., Jacob D. Jaffe</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>2021</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>data-paper</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Scientific Data</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41597-021-01008-4</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>17</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>2021: 1; 2022: 5; 2023: 5; 2024: 3; 2025: 2; 2026: 1</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -844,33 +905,38 @@
           <t>A proteomic atlas of senescence-associated secretomes for aging biomarker development</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Nathan Basisty, Abhijit Kale, Ok Hee Jeon, Chisaka Kuehnemann, Therese Payne, ..., Birgit Schilling</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>2020</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>PLoS Biology</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://doi.org/10.1371/journal.pbio.3000599</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>1312</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>2019: 3; 2020: 83; 2021: 183; 2022: 213; 2023: 222; 2024: 246; 2025: 229; 2026: 133</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -878,33 +944,38 @@
           <t>Skyline for Small Molecules: A Unifying Software Package for Quantitative Metabolomics</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kendra J. Adams, Brian Pratt, Neelanjan Bose, Laura G. Dubois, Lisa St. John‐Williams, ..., Alzheimer’s Disease Metabolomics Consortium</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>2020</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.jproteome.9b00640</t>
         </is>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>637</v>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>2020: 12; 2021: 57; 2022: 76; 2023: 117; 2024: 157; 2025: 140; 2026: 77</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -912,33 +983,38 @@
           <t>Audit logs to enforce document integrity in Skyline and Panorama</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tobias Rohde, Rita Chupalov, Nicholas Shulman, Vagisha Sharma, Josh Eckels, ..., Brendan MacLean</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
         <v>2020</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>Bioinformatics</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/bioinformatics/btaa547</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>5</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>2021: 2; 2022: 1; 2024: 2</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -946,29 +1022,34 @@
           <t>The HUPO-PSI standardized spectral library format</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ralf Gabriels, Nuno Bandeira, Wout Bittremieux, Jeremy Carver, Chambers, Matthew, ..., Eric W. Deutsch</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
         <v>2020</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>conference-paper</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Ghent University Academic Bibliography (Ghent University)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>https://doi.org/10.5281/zenodo.3607178</t>
         </is>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>0</v>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -976,33 +1057,38 @@
           <t>The ProteomeXchange consortium in 2020: enabling ‘big data’ approaches in proteomics</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Eric W. Deutsch, Nuno Bandeira, Vagisha Sharma, Yasset Pérez‐Riverol, Jeremy Carver, ..., Juan Antonio Vizcaíno</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>2019</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>Nucleic Acids Research</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/nar/gkz984</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>778</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>2019: 2; 2020: 80; 2021: 159; 2022: 207; 2023: 159; 2024: 111; 2025: 50; 2026: 10</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1010,33 +1096,38 @@
           <t>A Proteomic Atlas of Senescence-Associated Secretomes for Aging Biomarker Development</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Nathan Basisty, Abhijit Kale, Ok‐Hee Jeon, Chisaka Kuehnemann, Therese Payne, ..., Birgit Schilling</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>2019</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>bioRxiv (Cold Spring Harbor Laboratory)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>https://doi.org/10.1101/604306</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>111</v>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>2019: 1; 2020: 10; 2021: 36; 2022: 21; 2023: 11; 2024: 21; 2025: 10; 2026: 1</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1044,33 +1135,38 @@
           <t>piNET: a versatile web platform for downstream analysis and visualization of proteomics data</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Behrouz Shamsaei, Szymon Chojnacki, Marcin Pilarczyk, Mehdi Fazel Najafabadi, Chuming Chen, ..., Jarek Meller</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>2019</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>bioRxiv (Cold Spring Harbor Laboratory)</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>https://doi.org/10.1101/607432</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>2</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>2020: 2</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1078,33 +1174,38 @@
           <t>Panorama Public: A Public Repository for Quantitative Data Sets Processed in Skyline</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vagisha Sharma, Josh Eckels, Birgit Schilling, Christina Ludwig, Jacob D. Jaffe, ..., Brendan MacLean</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
         <v>2018</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>Molecular &amp; Cellular Proteomics</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>https://doi.org/10.1074/mcp.ra117.000543</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>286</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>2014: 1; 2018: 9; 2019: 22; 2020: 40; 2021: 42; 2022: 39; 2023: 37; 2024: 42; 2025: 38; 2026: 16</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1112,33 +1213,38 @@
           <t>A Library of Phosphoproteomic and Chromatin Signatures for Characterizing Cellular Responses to Drug Perturbations</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Lev Litichevskiy, Ryan Peckner, Jennifer G. Abelin, Jacob K. Asiedu, Amanda L. Creech, ..., Jacob D. Jaffe</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
         <v>2018</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>Cell Systems</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cels.2018.03.012</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>96</v>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>2017: 3; 2018: 10; 2019: 15; 2020: 10; 2021: 17; 2022: 10; 2023: 10; 2024: 5; 2025: 13; 2026: 3</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1146,33 +1252,38 @@
           <t>A Library of Phosphoproteomic and Chromatin Signatures for Characterizing Cellular Responses to Drug Perturbations</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lev Litichevskiy, Ryan Peckner, Jennifer G. Abelin, Jacob K. Asiedu, Amanda L. Creech, ..., Jacob D. Jaffe</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
         <v>2017</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>bioRxiv (Cold Spring Harbor Laboratory)</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>https://doi.org/10.1101/185918</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>3</v>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>2017: 2; 2022: 1</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1180,33 +1291,38 @@
           <t>Using the CPTAC Assay Portal to Identify and Implement Highly Characterized Targeted Proteomics Assays</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Jeffrey R. Whiteaker, Goran N. Halusa, Andrew N. Hoofnagle, Vagisha Sharma, Brendan MacLean, ..., Amanda G. Paulovich</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>2016</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>book-chapter</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Methods in molecular biology</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/978-1-4939-3524-6_13</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>101</v>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>2016: 4; 2017: 4; 2018: 5; 2019: 3; 2020: 3; 2021: 6; 2022: 3; 2023: 5; 2024: 60; 2025: 4; 2026: 3</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1214,33 +1330,38 @@
           <t>An Automated Pipeline to Monitor System Performance in Liquid Chromatography–Tandem Mass Spectrometry Proteomic Experiments</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Michael S. Bereman, Joshua Beri, Vagisha Sharma, Cory Nathe, Josh Eckels, ..., Michael J. MacCoss</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
         <v>2016</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/acs.jproteome.6b00744</t>
         </is>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>74</v>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>2016: 1; 2017: 5; 2018: 14; 2019: 3; 2020: 11; 2021: 6; 2022: 8; 2023: 6; 2024: 11; 2025: 6; 2026: 3</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1248,33 +1369,38 @@
           <t>Visualization and Dissemination of Multidimensional Proteomics Data Comparing Protein Abundance During &lt;i&gt;Caenorhabditis elegans&lt;/i&gt; Development</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Michael Riffle, Gennifer E. Merrihew, Daniel Jaschob, Vagisha Sharma, Trisha N. Davis, ..., Michael J. MacCoss</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>2015</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
           <t>Journal of the American Society for Mass Spectrometry</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s13361-015-1193-z</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>7</v>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>2016: 2; 2018: 3; 2019: 1; 2024: 1</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1282,33 +1408,38 @@
           <t>CPTAC Assay Portal: a repository of targeted proteomic assays</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Jeffrey R. Whiteaker, Goran N. Halusa, Andrew N. Hoofnagle, Vagisha Sharma, Brendan MacLean, ..., Amanda G. Paulovich</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
         <v>2014</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
           <t>Nature Methods</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/nmeth.3002</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>265</v>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>2014: 4; 2015: 11; 2016: 17; 2017: 10; 2018: 16; 2019: 12; 2020: 16; 2021: 24; 2022: 36; 2023: 19; 2024: 75; 2025: 18; 2026: 7</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1316,33 +1447,38 @@
           <t>Panorama: A Targeted Proteomics Knowledge Base</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Vagisha Sharma, Josh Eckels, Greg Taylor, Nicholas Shulman, Andrew B. Stergachis, ..., Brendan MacLean</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
         <v>2014</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/pr5006636</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>237</v>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>2014: 4; 2015: 18; 2016: 24; 2017: 24; 2018: 27; 2019: 15; 2020: 26; 2021: 28; 2022: 17; 2023: 18; 2024: 18; 2025: 14; 2026: 4</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1350,33 +1486,38 @@
           <t>A framework for installable external tools in Skyline</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Daniel Broudy, Trevor Killeen, Meena Choi, Nicholas Shulman, D.R. Mani, ..., Brendan MacLean</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
         <v>2014</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D28" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
           <t>Bioinformatics</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/bioinformatics/btu148</t>
         </is>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>36</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>2014: 3; 2015: 5; 2016: 7; 2017: 4; 2018: 3; 2019: 3; 2020: 4; 2021: 2; 2023: 1; 2024: 4</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1384,33 +1525,38 @@
           <t>XLink-DB: Database and Software Tools for Storing and Visualizing Protein Interaction Topology Data</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Chunxiang Zheng, Chad R. Weisbrod, Juan D. Chavez, Jimmy K. Eng, Vagisha Sharma, ..., James E. Bruce</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
         <v>2013</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/pr301162j</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>50</v>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>2013: 3; 2014: 1; 2015: 5; 2016: 4; 2017: 4; 2018: 10; 2019: 5; 2020: 3; 2021: 5; 2022: 2; 2023: 5; 2024: 2; 2025: 1</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1418,33 +1564,38 @@
           <t>A Mass Spectrometry Proteomics Data Management Platform</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Vagisha Sharma, Jimmy K. Eng, Michael J. MacCoss, Michael Riffle</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
         <v>2012</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D30" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>Molecular &amp; Cellular Proteomics</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>https://doi.org/10.1074/mcp.o111.015149</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>41</v>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>2012: 1; 2013: 2; 2014: 4; 2015: 4; 2016: 5; 2017: 5; 2018: 3; 2019: 1; 2020: 1; 2021: 1; 2022: 2; 2023: 3; 2024: 3; 2025: 3; 2026: 3</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1452,29 +1603,34 @@
           <t>P1) Technology Development in a Multidisciplinary Center</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Trisha N. Davis, Daniel A. Skelly, Gennifer E. Merrihew, Michael Riffle, Sara J. Cooper, ..., Joshua M. Akey</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
         <v>2012</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D31" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
           <t>Europe PMC (PubMed Central)</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>http://europepmc.org/articles/PMC3630640</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>0</v>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1482,33 +1638,38 @@
           <t>Precursor Charge State Prediction for Electron Transfer Dissociation Tandem Mass Spectra</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Vagisha Sharma, Jimmy K. Eng, Sergey Feldman, Priska D. von Haller, Michael J. MacCoss, William Stafford Noble</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
         <v>2010</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D32" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
           <t>Journal of Proteome Research</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>https://doi.org/10.1021/pr1006685</t>
         </is>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>13</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>2012: 1; 2013: 3; 2016: 1; 2017: 2; 2019: 1; 2022: 1; 2024: 1; 2025: 2</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1516,33 +1677,38 @@
           <t>Corra: Computational framework and tools for LC-MS discovery and targeted mass spectrometry-based proteomics</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Mi‐Youn Brusniak, Bernd Bodenmiller, David Campbell, Kelly Cooke, James S. Eddes, ..., Julian D. Watts</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
         <v>2008</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>article</t>
-        </is>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
           <t>BMC Bioinformatics</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>https://doi.org/10.1186/1471-2105-9-542</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="G33" t="n">
         <v>74</v>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>2012: 7; 2013: 7; 2014: 7; 2015: 2; 2017: 1; 2018: 4; 2019: 1; 2020: 1; 2021: 3; 2022: 1; 2024: 1</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>